<commit_message>
Inicio da implementação de reescala
Antes de iniciar, foi necessário melhor as saída da melhor escala do tipo 1. Além disso, gráficos mais detalhados do melhor foram gerados. Iniciando o processamento da entrada: escala, dia e o nome do funcionário que faltou.
Refatoração de alguns módulos.
</commit_message>
<xml_diff>
--- a/Testes/Teste mutação/Teste2/3_melhor_escala_global.xlsx
+++ b/Testes/Teste mutação/Teste2/3_melhor_escala_global.xlsx
@@ -27,7 +27,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,26 +42,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0090EE90"/>
-        <bgColor rgb="0090EE90"/>
+        <fgColor rgb="00B9FF80"/>
+        <bgColor rgb="00B9FF80"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFB6C6"/>
-        <bgColor rgb="00FFB6C6"/>
+        <fgColor rgb="00F7FFC9"/>
+        <bgColor rgb="00F7FFC9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -100,10 +100,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -469,14 +468,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH54"/>
+  <dimension ref="A1:AI52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
@@ -505,7 +504,9 @@
     <col width="8" customWidth="1" min="31" max="31"/>
     <col width="8" customWidth="1" min="32" max="32"/>
     <col width="8" customWidth="1" min="33" max="33"/>
-    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="8" customWidth="1" min="34" max="34"/>
+    <col width="8" customWidth="1" min="35" max="35"/>
+    <col width="8" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,162 +522,167 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Início licença</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fim licença</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Último dia do mês anterior</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Dia 1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Dia 2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Dia 3</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dia 4</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Dia 5</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dia 6</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dia 7</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dia 8</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Dia 9</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Dia 10</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Dia 11</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Dia 12</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Dia 13</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Dia 14</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Dia 15</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Dia 16</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Dia 17</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Dia 18</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Dia 19</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Dia 20</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Dia 21</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Dia 22</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Dia 23</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Dia 24</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Dia 25</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Dia 26</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Dia 27</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Dia 28</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Dia 29</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Dia 30</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>Total dias escalados</t>
         </is>
       </c>
     </row>
@@ -694,10 +700,10 @@
       <c r="C2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="5" t="n">
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="4" t="n">
@@ -766,11 +772,11 @@
       <c r="AA2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="4" t="n">
-        <v>1</v>
+      <c r="AB2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -784,9 +790,11 @@
       <c r="AG2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH2" s="6">
-        <f>SUM(D2:AG2)</f>
-        <v/>
+      <c r="AH2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -801,12 +809,12 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="5" t="n">
@@ -815,87 +823,89 @@
       <c r="G3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="5" t="n">
+      <c r="H3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="6" t="n">
         <v>0</v>
       </c>
       <c r="AG3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH3" s="6">
-        <f>SUM(D3:AG3)</f>
-        <v/>
+      <c r="AH3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -910,12 +920,12 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="5" t="n">
@@ -987,11 +997,11 @@
       <c r="AB4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="4" t="n">
-        <v>1</v>
+      <c r="AC4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD4" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AE4" s="5" t="n">
         <v>0</v>
@@ -1002,9 +1012,11 @@
       <c r="AG4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="6">
-        <f>SUM(D4:AG4)</f>
-        <v/>
+      <c r="AH4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI4" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1019,12 +1031,12 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
@@ -1042,11 +1054,11 @@
       <c r="J5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>1</v>
+      <c r="K5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>0</v>
@@ -1063,20 +1075,20 @@
       <c r="Q5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4" t="n">
-        <v>1</v>
+      <c r="R5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="4" t="n">
-        <v>1</v>
+      <c r="U5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V5" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="W5" s="5" t="n">
         <v>0</v>
@@ -1099,11 +1111,11 @@
       <c r="AC5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AD5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="4" t="n">
-        <v>1</v>
+      <c r="AD5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE5" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AF5" s="5" t="n">
         <v>0</v>
@@ -1111,9 +1123,11 @@
       <c r="AG5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH5" s="6">
-        <f>SUM(D5:AG5)</f>
-        <v/>
+      <c r="AH5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1128,16 +1142,16 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>0</v>
@@ -1220,9 +1234,11 @@
       <c r="AG6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH6" s="6">
-        <f>SUM(D6:AG6)</f>
-        <v/>
+      <c r="AH6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1237,12 +1253,12 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="5" t="n">
@@ -1266,11 +1282,11 @@
       <c r="L7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="4" t="n">
-        <v>1</v>
+      <c r="M7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="O7" s="5" t="n">
         <v>0</v>
@@ -1329,9 +1345,11 @@
       <c r="AG7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH7" s="6">
-        <f>SUM(D7:AG7)</f>
-        <v/>
+      <c r="AH7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1346,22 +1364,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>1</v>
+      <c r="G8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>0</v>
@@ -1396,20 +1414,20 @@
       <c r="S8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>1</v>
+      <c r="T8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="V8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="W8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" s="4" t="n">
-        <v>1</v>
+      <c r="W8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Y8" s="5" t="n">
         <v>0</v>
@@ -1438,9 +1456,11 @@
       <c r="AG8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH8" s="6">
-        <f>SUM(D8:AG8)</f>
-        <v/>
+      <c r="AH8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI8" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1457,17 +1477,17 @@
       <c r="C9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>1</v>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
         <v>0</v>
@@ -1508,11 +1528,11 @@
       <c r="T9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" s="4" t="n">
-        <v>1</v>
+      <c r="U9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="W9" s="5" t="n">
         <v>0</v>
@@ -1547,9 +1567,11 @@
       <c r="AG9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH9" s="6">
-        <f>SUM(D9:AG9)</f>
-        <v/>
+      <c r="AH9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1564,12 +1586,12 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="5" t="n">
@@ -1605,11 +1627,11 @@
       <c r="P10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Q10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>1</v>
+      <c r="Q10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="S10" s="5" t="n">
         <v>0</v>
@@ -1626,11 +1648,11 @@
       <c r="W10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="X10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="4" t="n">
-        <v>1</v>
+      <c r="X10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Z10" s="5" t="n">
         <v>0</v>
@@ -1656,9 +1678,11 @@
       <c r="AG10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH10" s="6">
-        <f>SUM(D10:AG10)</f>
-        <v/>
+      <c r="AH10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI10" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1675,17 +1699,17 @@
       <c r="C11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>1</v>
+      <c r="D11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>0</v>
@@ -1708,11 +1732,11 @@
       <c r="N11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="4" t="n">
-        <v>1</v>
+      <c r="O11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1723,11 +1747,11 @@
       <c r="S11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="4" t="n">
-        <v>1</v>
+      <c r="T11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="V11" s="5" t="n">
         <v>0</v>
@@ -1765,9 +1789,11 @@
       <c r="AG11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH11" s="6">
-        <f>SUM(D11:AG11)</f>
-        <v/>
+      <c r="AH11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1784,10 +1810,10 @@
       <c r="C12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="5" t="n">
+      <c r="D12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="4" t="n">
@@ -1802,11 +1828,11 @@
       <c r="I12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>1</v>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L12" s="5" t="n">
         <v>0</v>
@@ -1841,11 +1867,11 @@
       <c r="V12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="W12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" s="4" t="n">
-        <v>1</v>
+      <c r="W12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X12" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Y12" s="5" t="n">
         <v>0</v>
@@ -1874,9 +1900,11 @@
       <c r="AG12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH12" s="6">
-        <f>SUM(D12:AG12)</f>
-        <v/>
+      <c r="AH12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI12" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1891,12 +1919,12 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
@@ -1926,11 +1954,11 @@
       <c r="N13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="4" t="n">
-        <v>1</v>
+      <c r="O13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1953,11 +1981,11 @@
       <c r="W13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="X13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="4" t="n">
-        <v>1</v>
+      <c r="X13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Z13" s="5" t="n">
         <v>0</v>
@@ -1983,9 +2011,11 @@
       <c r="AG13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH13" s="6">
-        <f>SUM(D13:AG13)</f>
-        <v/>
+      <c r="AH13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI13" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2002,55 +2032,55 @@
       <c r="C14" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T14" s="5" t="n">
+      <c r="D14" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="6" t="n">
         <v>0</v>
       </c>
       <c r="U14" s="4" t="n">
@@ -2083,18 +2113,20 @@
       <c r="AD14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="4" t="n">
-        <v>1</v>
+      <c r="AE14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF14" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AG14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH14" s="6">
-        <f>SUM(D14:AG14)</f>
-        <v/>
+      <c r="AH14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI14" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2109,22 +2141,22 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>1</v>
+      <c r="G15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>0</v>
@@ -2159,11 +2191,11 @@
       <c r="S15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="4" t="n">
-        <v>1</v>
+      <c r="T15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="V15" s="5" t="n">
         <v>0</v>
@@ -2201,9 +2233,11 @@
       <c r="AG15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH15" s="6">
-        <f>SUM(D15:AG15)</f>
-        <v/>
+      <c r="AH15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2220,10 +2254,10 @@
       <c r="C16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5" t="n">
+      <c r="D16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="4" t="n">
@@ -2250,11 +2284,11 @@
       <c r="M16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="4" t="n">
-        <v>1</v>
+      <c r="N16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="P16" s="5" t="n">
         <v>0</v>
@@ -2310,9 +2344,11 @@
       <c r="AG16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH16" s="6">
-        <f>SUM(D16:AG16)</f>
-        <v/>
+      <c r="AH16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI16" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2327,12 +2363,12 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="5" t="n">
@@ -2404,11 +2440,11 @@
       <c r="AB17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD17" s="4" t="n">
-        <v>1</v>
+      <c r="AC17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD17" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AE17" s="5" t="n">
         <v>0</v>
@@ -2419,9 +2455,11 @@
       <c r="AG17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH17" s="6">
-        <f>SUM(D17:AG17)</f>
-        <v/>
+      <c r="AH17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI17" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2438,10 +2476,10 @@
       <c r="C18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="5" t="n">
+      <c r="D18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="4" t="n">
@@ -2462,11 +2500,11 @@
       <c r="K18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="N18" s="5" t="n">
         <v>0</v>
@@ -2483,11 +2521,11 @@
       <c r="R18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T18" s="4" t="n">
-        <v>1</v>
+      <c r="S18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U18" s="5" t="n">
         <v>0</v>
@@ -2528,9 +2566,11 @@
       <c r="AG18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH18" s="6">
-        <f>SUM(D18:AG18)</f>
-        <v/>
+      <c r="AH18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI18" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -2545,12 +2585,12 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="5" t="n">
@@ -2562,11 +2602,11 @@
       <c r="H19" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>1</v>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>0</v>
@@ -2613,11 +2653,11 @@
       <c r="Y19" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="4" t="n">
-        <v>1</v>
+      <c r="Z19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA19" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AB19" s="5" t="n">
         <v>0</v>
@@ -2637,9 +2677,11 @@
       <c r="AG19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH19" s="6">
-        <f>SUM(D19:AG19)</f>
-        <v/>
+      <c r="AH19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2654,12 +2696,12 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="5" t="n">
@@ -2701,11 +2743,11 @@
       <c r="R20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>1</v>
+      <c r="S20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U20" s="5" t="n">
         <v>0</v>
@@ -2746,9 +2788,11 @@
       <c r="AG20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH20" s="6">
-        <f>SUM(D20:AG20)</f>
-        <v/>
+      <c r="AH20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI20" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -2763,12 +2807,12 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="5" t="n">
@@ -2855,9 +2899,11 @@
       <c r="AG21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH21" s="6">
-        <f>SUM(D21:AG21)</f>
-        <v/>
+      <c r="AH21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI21" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2872,12 +2918,12 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="5" t="n">
@@ -2895,11 +2941,11 @@
       <c r="J22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>1</v>
+      <c r="K22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="M22" s="5" t="n">
         <v>0</v>
@@ -2910,11 +2956,11 @@
       <c r="O22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>1</v>
+      <c r="P22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R22" s="5" t="n">
         <v>0</v>
@@ -2964,9 +3010,11 @@
       <c r="AG22" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH22" s="6">
-        <f>SUM(D22:AG22)</f>
-        <v/>
+      <c r="AH22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI22" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2983,11 +3031,11 @@
       <c r="C23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>1</v>
+      <c r="D23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>0</v>
@@ -3073,9 +3121,11 @@
       <c r="AG23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH23" s="6">
-        <f>SUM(D23:AG23)</f>
-        <v/>
+      <c r="AH23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI23" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -3092,17 +3142,17 @@
       <c r="C24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>1</v>
+      <c r="D24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H24" s="5" t="n">
         <v>0</v>
@@ -3182,9 +3232,11 @@
       <c r="AG24" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH24" s="6">
-        <f>SUM(D24:AG24)</f>
-        <v/>
+      <c r="AH24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI24" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -3199,22 +3251,22 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>1</v>
+      <c r="G25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="I25" s="5" t="n">
         <v>0</v>
@@ -3237,11 +3289,11 @@
       <c r="O25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="4" t="n">
-        <v>1</v>
+      <c r="P25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R25" s="5" t="n">
         <v>0</v>
@@ -3264,11 +3316,11 @@
       <c r="X25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z25" s="4" t="n">
-        <v>1</v>
+      <c r="Y25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z25" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AA25" s="5" t="n">
         <v>0</v>
@@ -3291,9 +3343,11 @@
       <c r="AG25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH25" s="6">
-        <f>SUM(D25:AG25)</f>
-        <v/>
+      <c r="AH25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI25" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3308,12 +3362,12 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="5" t="n">
@@ -3325,11 +3379,11 @@
       <c r="H26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="4" t="n">
-        <v>1</v>
+      <c r="I26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="K26" s="5" t="n">
         <v>0</v>
@@ -3376,11 +3430,11 @@
       <c r="Y26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA26" s="4" t="n">
-        <v>1</v>
+      <c r="Z26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA26" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AB26" s="5" t="n">
         <v>0</v>
@@ -3400,9 +3454,11 @@
       <c r="AG26" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH26" s="6">
-        <f>SUM(D26:AG26)</f>
-        <v/>
+      <c r="AH26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI26" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -3417,12 +3473,12 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="5" t="n">
@@ -3440,20 +3496,20 @@
       <c r="J27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="4" t="n">
-        <v>1</v>
+      <c r="K27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="M27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="4" t="n">
-        <v>1</v>
+      <c r="N27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="P27" s="5" t="n">
         <v>0</v>
@@ -3494,11 +3550,11 @@
       <c r="AB27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD27" s="4" t="n">
-        <v>1</v>
+      <c r="AC27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD27" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AE27" s="5" t="n">
         <v>0</v>
@@ -3509,9 +3565,11 @@
       <c r="AG27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH27" s="6">
-        <f>SUM(D27:AG27)</f>
-        <v/>
+      <c r="AH27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI27" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3526,12 +3584,12 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="5" t="n">
@@ -3618,9 +3676,11 @@
       <c r="AG28" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH28" s="6">
-        <f>SUM(D28:AG28)</f>
-        <v/>
+      <c r="AH28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI28" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -3637,17 +3697,17 @@
       <c r="C29" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="4" t="n">
-        <v>1</v>
+      <c r="D29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H29" s="5" t="n">
         <v>0</v>
@@ -3682,11 +3742,11 @@
       <c r="R29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" s="4" t="n">
-        <v>1</v>
+      <c r="S29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T29" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U29" s="5" t="n">
         <v>0</v>
@@ -3715,11 +3775,11 @@
       <c r="AC29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AD29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE29" s="4" t="n">
-        <v>1</v>
+      <c r="AD29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE29" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AF29" s="5" t="n">
         <v>0</v>
@@ -3727,9 +3787,11 @@
       <c r="AG29" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH29" s="6">
-        <f>SUM(D29:AG29)</f>
-        <v/>
+      <c r="AH29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -3746,10 +3808,10 @@
       <c r="C30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="5" t="n">
+      <c r="D30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="4" t="n">
@@ -3812,11 +3874,11 @@
       <c r="Y30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA30" s="4" t="n">
-        <v>1</v>
+      <c r="Z30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA30" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AB30" s="5" t="n">
         <v>0</v>
@@ -3836,9 +3898,11 @@
       <c r="AG30" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH30" s="6">
-        <f>SUM(D30:AG30)</f>
-        <v/>
+      <c r="AH30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI30" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -3855,10 +3919,10 @@
       <c r="C31" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="5" t="n">
+      <c r="D31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="4" t="n">
@@ -3873,11 +3937,11 @@
       <c r="I31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="4" t="n">
-        <v>1</v>
+      <c r="J31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L31" s="5" t="n">
         <v>0</v>
@@ -3888,11 +3952,11 @@
       <c r="N31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="4" t="n">
-        <v>1</v>
+      <c r="O31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Q31" s="5" t="n">
         <v>0</v>
@@ -3909,11 +3973,11 @@
       <c r="U31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="V31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W31" s="4" t="n">
-        <v>1</v>
+      <c r="V31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W31" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="X31" s="5" t="n">
         <v>0</v>
@@ -3945,9 +4009,11 @@
       <c r="AG31" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH31" s="6">
-        <f>SUM(D31:AG31)</f>
-        <v/>
+      <c r="AH31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI31" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -3964,10 +4030,10 @@
       <c r="C32" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="5" t="n">
+      <c r="D32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F32" s="4" t="n">
@@ -4054,9 +4120,11 @@
       <c r="AG32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH32" s="6">
-        <f>SUM(D32:AG32)</f>
-        <v/>
+      <c r="AH32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI32" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -4071,12 +4139,12 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="5" t="n">
@@ -4130,11 +4198,11 @@
       <c r="V33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="W33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X33" s="4" t="n">
-        <v>1</v>
+      <c r="W33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X33" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Y33" s="5" t="n">
         <v>0</v>
@@ -4163,9 +4231,11 @@
       <c r="AG33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH33" s="6">
-        <f>SUM(D33:AG33)</f>
-        <v/>
+      <c r="AH33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI33" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -4182,10 +4252,10 @@
       <c r="C34" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="5" t="n">
+      <c r="D34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="4" t="n">
@@ -4242,20 +4312,20 @@
       <c r="W34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="X34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y34" s="4" t="n">
-        <v>1</v>
+      <c r="X34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Z34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB34" s="4" t="n">
-        <v>1</v>
+      <c r="AA34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AC34" s="5" t="n">
         <v>0</v>
@@ -4272,9 +4342,11 @@
       <c r="AG34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH34" s="6">
-        <f>SUM(D34:AG34)</f>
-        <v/>
+      <c r="AH34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI34" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -4291,10 +4363,10 @@
       <c r="C35" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="5" t="n">
+      <c r="D35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="4" t="n">
@@ -4345,29 +4417,29 @@
       <c r="U35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="V35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W35" s="4" t="n">
-        <v>1</v>
+      <c r="V35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W35" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="X35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z35" s="4" t="n">
-        <v>1</v>
+      <c r="Y35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z35" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AA35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC35" s="4" t="n">
-        <v>1</v>
+      <c r="AB35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC35" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AD35" s="5" t="n">
         <v>0</v>
@@ -4381,9 +4453,11 @@
       <c r="AG35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH35" s="6">
-        <f>SUM(D35:AG35)</f>
-        <v/>
+      <c r="AH35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI35" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -4400,10 +4474,10 @@
       <c r="C36" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="5" t="n">
+      <c r="D36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="4" t="n">
@@ -4412,11 +4486,11 @@
       <c r="G36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="4" t="n">
-        <v>1</v>
+      <c r="H36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0</v>
@@ -4481,18 +4555,20 @@
       <c r="AD36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF36" s="4" t="n">
-        <v>1</v>
+      <c r="AE36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF36" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AG36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH36" s="6">
-        <f>SUM(D36:AG36)</f>
-        <v/>
+      <c r="AH36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI36" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -4507,22 +4583,22 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="4" t="n">
-        <v>1</v>
+      <c r="G37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="I37" s="5" t="n">
         <v>0</v>
@@ -4599,9 +4675,11 @@
       <c r="AG37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH37" s="6">
-        <f>SUM(D37:AG37)</f>
-        <v/>
+      <c r="AH37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI37" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -4618,10 +4696,10 @@
       <c r="C38" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="5" t="n">
+      <c r="D38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="4" t="n">
@@ -4654,11 +4732,11 @@
       <c r="O38" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="4" t="n">
-        <v>1</v>
+      <c r="P38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="R38" s="5" t="n">
         <v>0</v>
@@ -4708,9 +4786,11 @@
       <c r="AG38" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH38" s="6">
-        <f>SUM(D38:AG38)</f>
-        <v/>
+      <c r="AH38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI38" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -4727,10 +4807,10 @@
       <c r="C39" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D39" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="5" t="n">
+      <c r="D39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="4" t="n">
@@ -4739,11 +4819,11 @@
       <c r="G39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="4" t="n">
-        <v>1</v>
+      <c r="H39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J39" s="5" t="n">
         <v>0</v>
@@ -4754,11 +4834,11 @@
       <c r="L39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="4" t="n">
-        <v>1</v>
+      <c r="M39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N39" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="O39" s="5" t="n">
         <v>0</v>
@@ -4817,9 +4897,11 @@
       <c r="AG39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH39" s="6">
-        <f>SUM(D39:AG39)</f>
-        <v/>
+      <c r="AH39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI39" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4834,16 +4916,16 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G40" s="5" t="n">
         <v>0</v>
@@ -4860,20 +4942,20 @@
       <c r="K40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" s="4" t="n">
-        <v>1</v>
+      <c r="L40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="N40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="4" t="n">
-        <v>1</v>
+      <c r="O40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P40" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Q40" s="5" t="n">
         <v>0</v>
@@ -4926,9 +5008,11 @@
       <c r="AG40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH40" s="6">
-        <f>SUM(D40:AG40)</f>
-        <v/>
+      <c r="AH40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI40" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4945,11 +5029,11 @@
       <c r="C41" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="4" t="n">
-        <v>1</v>
+      <c r="D41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F41" s="5" t="n">
         <v>0</v>
@@ -4966,11 +5050,11 @@
       <c r="J41" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" s="4" t="n">
-        <v>1</v>
+      <c r="K41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L41" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="M41" s="5" t="n">
         <v>0</v>
@@ -5029,15 +5113,17 @@
       <c r="AE41" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AF41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH41" s="6">
-        <f>SUM(D41:AG41)</f>
-        <v/>
+      <c r="AF41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI41" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -5054,10 +5140,10 @@
       <c r="C42" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="5" t="n">
+      <c r="D42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="4" t="n">
@@ -5144,9 +5230,11 @@
       <c r="AG42" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH42" s="6">
-        <f>SUM(D42:AG42)</f>
-        <v/>
+      <c r="AH42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI42" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -5161,12 +5249,12 @@
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="5" t="n">
@@ -5238,11 +5326,11 @@
       <c r="AB43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD43" s="4" t="n">
-        <v>1</v>
+      <c r="AC43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD43" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AE43" s="5" t="n">
         <v>0</v>
@@ -5253,9 +5341,11 @@
       <c r="AG43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH43" s="6">
-        <f>SUM(D43:AG43)</f>
-        <v/>
+      <c r="AH43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI43" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -5270,12 +5360,12 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="5" t="n">
@@ -5362,9 +5452,11 @@
       <c r="AG44" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH44" s="6">
-        <f>SUM(D44:AG44)</f>
-        <v/>
+      <c r="AH44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI44" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -5381,10 +5473,10 @@
       <c r="C45" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="5" t="n">
+      <c r="D45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="4" t="n">
@@ -5411,11 +5503,11 @@
       <c r="M45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O45" s="4" t="n">
-        <v>1</v>
+      <c r="N45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O45" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="P45" s="5" t="n">
         <v>0</v>
@@ -5444,11 +5536,11 @@
       <c r="X45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z45" s="4" t="n">
-        <v>1</v>
+      <c r="Y45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z45" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AA45" s="5" t="n">
         <v>0</v>
@@ -5459,11 +5551,11 @@
       <c r="AC45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AD45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE45" s="4" t="n">
-        <v>1</v>
+      <c r="AD45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE45" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AF45" s="5" t="n">
         <v>0</v>
@@ -5471,9 +5563,11 @@
       <c r="AG45" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH45" s="6">
-        <f>SUM(D45:AG45)</f>
-        <v/>
+      <c r="AH45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI45" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -5488,16 +5582,16 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G46" s="5" t="n">
         <v>0</v>
@@ -5580,9 +5674,11 @@
       <c r="AG46" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH46" s="6">
-        <f>SUM(D46:AG46)</f>
-        <v/>
+      <c r="AH46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI46" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -5597,16 +5693,16 @@
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>0</v>
@@ -5623,11 +5719,11 @@
       <c r="K47" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M47" s="4" t="n">
-        <v>1</v>
+      <c r="L47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="N47" s="5" t="n">
         <v>0</v>
@@ -5689,9 +5785,11 @@
       <c r="AG47" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH47" s="6">
-        <f>SUM(D47:AG47)</f>
-        <v/>
+      <c r="AH47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI47" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -5706,82 +5804,82 @@
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S48" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U48" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W48" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y48" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA48" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB48" s="4" t="n">
-        <v>1</v>
+        <v>22</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="V48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="X48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB48" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AC48" s="5" t="n">
         <v>0</v>
@@ -5798,9 +5896,11 @@
       <c r="AG48" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH48" s="6">
-        <f>SUM(D48:AG48)</f>
-        <v/>
+      <c r="AH48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI48" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -5817,10 +5917,10 @@
       <c r="C49" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="5" t="n">
+      <c r="D49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F49" s="4" t="n">
@@ -5829,11 +5929,11 @@
       <c r="G49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" s="4" t="n">
-        <v>1</v>
+      <c r="H49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J49" s="5" t="n">
         <v>0</v>
@@ -5862,11 +5962,11 @@
       <c r="R49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T49" s="4" t="n">
-        <v>1</v>
+      <c r="S49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T49" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U49" s="5" t="n">
         <v>0</v>
@@ -5907,9 +6007,11 @@
       <c r="AG49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH49" s="6">
-        <f>SUM(D49:AG49)</f>
-        <v/>
+      <c r="AH49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI49" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -5926,10 +6028,10 @@
       <c r="C50" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="5" t="n">
+      <c r="D50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="4" t="n">
@@ -5998,11 +6100,11 @@
       <c r="AA50" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC50" s="4" t="n">
-        <v>1</v>
+      <c r="AB50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC50" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AD50" s="5" t="n">
         <v>0</v>
@@ -6016,9 +6118,11 @@
       <c r="AG50" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH50" s="6">
-        <f>SUM(D50:AG50)</f>
-        <v/>
+      <c r="AH50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI50" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -6035,10 +6139,10 @@
       <c r="C51" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D51" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="5" t="n">
+      <c r="D51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F51" s="4" t="n">
@@ -6053,11 +6157,11 @@
       <c r="I51" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J51" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" s="4" t="n">
-        <v>1</v>
+      <c r="J51" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L51" s="5" t="n">
         <v>0</v>
@@ -6125,9 +6229,11 @@
       <c r="AG51" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="AH51" s="6">
-        <f>SUM(D51:AG51)</f>
-        <v/>
+      <c r="AH51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI51" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -6144,10 +6250,10 @@
       <c r="C52" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D52" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="5" t="n">
+      <c r="D52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F52" s="4" t="n">
@@ -6234,263 +6340,11 @@
       <c r="AG52" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH52" s="6">
-        <f>SUM(D52:AG52)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>Total de farmacêuticos:</t>
-        </is>
-      </c>
-      <c r="D53" s="6">
-        <f>SUM(D2:D4)</f>
-        <v/>
-      </c>
-      <c r="E53" s="6">
-        <f>SUM(E2:E4)</f>
-        <v/>
-      </c>
-      <c r="F53" s="6">
-        <f>SUM(F2:F4)</f>
-        <v/>
-      </c>
-      <c r="G53" s="6">
-        <f>SUM(G2:G4)</f>
-        <v/>
-      </c>
-      <c r="H53" s="6">
-        <f>SUM(H2:H4)</f>
-        <v/>
-      </c>
-      <c r="I53" s="6">
-        <f>SUM(I2:I4)</f>
-        <v/>
-      </c>
-      <c r="J53" s="6">
-        <f>SUM(J2:J4)</f>
-        <v/>
-      </c>
-      <c r="K53" s="6">
-        <f>SUM(K2:K4)</f>
-        <v/>
-      </c>
-      <c r="L53" s="6">
-        <f>SUM(L2:L4)</f>
-        <v/>
-      </c>
-      <c r="M53" s="6">
-        <f>SUM(M2:M4)</f>
-        <v/>
-      </c>
-      <c r="N53" s="6">
-        <f>SUM(N2:N4)</f>
-        <v/>
-      </c>
-      <c r="O53" s="6">
-        <f>SUM(O2:O4)</f>
-        <v/>
-      </c>
-      <c r="P53" s="6">
-        <f>SUM(P2:P4)</f>
-        <v/>
-      </c>
-      <c r="Q53" s="6">
-        <f>SUM(Q2:Q4)</f>
-        <v/>
-      </c>
-      <c r="R53" s="6">
-        <f>SUM(R2:R4)</f>
-        <v/>
-      </c>
-      <c r="S53" s="6">
-        <f>SUM(S2:S4)</f>
-        <v/>
-      </c>
-      <c r="T53" s="6">
-        <f>SUM(T2:T4)</f>
-        <v/>
-      </c>
-      <c r="U53" s="6">
-        <f>SUM(U2:U4)</f>
-        <v/>
-      </c>
-      <c r="V53" s="6">
-        <f>SUM(V2:V4)</f>
-        <v/>
-      </c>
-      <c r="W53" s="6">
-        <f>SUM(W2:W4)</f>
-        <v/>
-      </c>
-      <c r="X53" s="6">
-        <f>SUM(X2:X4)</f>
-        <v/>
-      </c>
-      <c r="Y53" s="6">
-        <f>SUM(Y2:Y4)</f>
-        <v/>
-      </c>
-      <c r="Z53" s="6">
-        <f>SUM(Z2:Z4)</f>
-        <v/>
-      </c>
-      <c r="AA53" s="6">
-        <f>SUM(AA2:AA4)</f>
-        <v/>
-      </c>
-      <c r="AB53" s="6">
-        <f>SUM(AB2:AB4)</f>
-        <v/>
-      </c>
-      <c r="AC53" s="6">
-        <f>SUM(AC2:AC4)</f>
-        <v/>
-      </c>
-      <c r="AD53" s="6">
-        <f>SUM(AD2:AD4)</f>
-        <v/>
-      </c>
-      <c r="AE53" s="6">
-        <f>SUM(AE2:AE4)</f>
-        <v/>
-      </c>
-      <c r="AF53" s="6">
-        <f>SUM(AF2:AF4)</f>
-        <v/>
-      </c>
-      <c r="AG53" s="6">
-        <f>SUM(AG2:AG4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>Total de auxiliares:</t>
-        </is>
-      </c>
-      <c r="D54" s="6">
-        <f>SUM(D5:D52)</f>
-        <v/>
-      </c>
-      <c r="E54" s="6">
-        <f>SUM(E5:E52)</f>
-        <v/>
-      </c>
-      <c r="F54" s="6">
-        <f>SUM(F5:F52)</f>
-        <v/>
-      </c>
-      <c r="G54" s="6">
-        <f>SUM(G5:G52)</f>
-        <v/>
-      </c>
-      <c r="H54" s="6">
-        <f>SUM(H5:H52)</f>
-        <v/>
-      </c>
-      <c r="I54" s="6">
-        <f>SUM(I5:I52)</f>
-        <v/>
-      </c>
-      <c r="J54" s="6">
-        <f>SUM(J5:J52)</f>
-        <v/>
-      </c>
-      <c r="K54" s="6">
-        <f>SUM(K5:K52)</f>
-        <v/>
-      </c>
-      <c r="L54" s="6">
-        <f>SUM(L5:L52)</f>
-        <v/>
-      </c>
-      <c r="M54" s="6">
-        <f>SUM(M5:M52)</f>
-        <v/>
-      </c>
-      <c r="N54" s="6">
-        <f>SUM(N5:N52)</f>
-        <v/>
-      </c>
-      <c r="O54" s="6">
-        <f>SUM(O5:O52)</f>
-        <v/>
-      </c>
-      <c r="P54" s="6">
-        <f>SUM(P5:P52)</f>
-        <v/>
-      </c>
-      <c r="Q54" s="6">
-        <f>SUM(Q5:Q52)</f>
-        <v/>
-      </c>
-      <c r="R54" s="6">
-        <f>SUM(R5:R52)</f>
-        <v/>
-      </c>
-      <c r="S54" s="6">
-        <f>SUM(S5:S52)</f>
-        <v/>
-      </c>
-      <c r="T54" s="6">
-        <f>SUM(T5:T52)</f>
-        <v/>
-      </c>
-      <c r="U54" s="6">
-        <f>SUM(U5:U52)</f>
-        <v/>
-      </c>
-      <c r="V54" s="6">
-        <f>SUM(V5:V52)</f>
-        <v/>
-      </c>
-      <c r="W54" s="6">
-        <f>SUM(W5:W52)</f>
-        <v/>
-      </c>
-      <c r="X54" s="6">
-        <f>SUM(X5:X52)</f>
-        <v/>
-      </c>
-      <c r="Y54" s="6">
-        <f>SUM(Y5:Y52)</f>
-        <v/>
-      </c>
-      <c r="Z54" s="6">
-        <f>SUM(Z5:Z52)</f>
-        <v/>
-      </c>
-      <c r="AA54" s="6">
-        <f>SUM(AA5:AA52)</f>
-        <v/>
-      </c>
-      <c r="AB54" s="6">
-        <f>SUM(AB5:AB52)</f>
-        <v/>
-      </c>
-      <c r="AC54" s="6">
-        <f>SUM(AC5:AC52)</f>
-        <v/>
-      </c>
-      <c r="AD54" s="6">
-        <f>SUM(AD5:AD52)</f>
-        <v/>
-      </c>
-      <c r="AE54" s="6">
-        <f>SUM(AE5:AE52)</f>
-        <v/>
-      </c>
-      <c r="AF54" s="6">
-        <f>SUM(AF5:AF52)</f>
-        <v/>
-      </c>
-      <c r="AG54" s="6">
-        <f>SUM(AG5:AG52)</f>
-        <v/>
+      <c r="AH52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI52" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>